<commit_message>
chore(data): daily refresh of list-source downloads
Updated: 2026-05-09T00:29:59+00:00
Total: 8, Success: 8, Failures: 0
</commit_message>
<xml_diff>
--- a/data/downloads/fatf-jurisdictions.xlsx
+++ b/data/downloads/fatf-jurisdictions.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-08T15:48:20+00:00</t>
+          <t>2026-05-09T00:27:21+00:00</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -945,7 +945,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Namibia</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Namibia</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Angola</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Angola</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Yemen</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Syria</t>
+          <t>Haiti</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Syria</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Yemen</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">

</xml_diff>